<commit_message>
Alteração matriz de requisitos original recuperada
Alteração da matriz de requisitos com base na copia original, recuperada.
</commit_message>
<xml_diff>
--- a/Documentacao_Engenharia/Lista_Requisitos_do_projeto_Estacionamento.xlsx
+++ b/Documentacao_Engenharia/Lista_Requisitos_do_projeto_Estacionamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{66B3DA27-E4C0-4B56-B56F-4028382647F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB79E335-D5B5-478E-A904-E255B89EEAD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5ECE2E23-00F7-44A7-9D17-79983676019F}"/>
   </bookViews>
@@ -50,20 +50,65 @@
     <t>Descrição das regras de domínio</t>
   </si>
   <si>
-    <t>*Legenda: Rf = Requisito não funcional</t>
+    <t>id*</t>
   </si>
   <si>
-    <t>id*</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*Legenda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rf = Requisito não funcional</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -84,7 +129,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.249977111117893"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -116,10 +161,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -465,18 +511,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
-        <v>3</v>
+      <c r="A2" s="4" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>1</v>

</xml_diff>